<commit_message>
回代 shared 0921 + 修复 SC 占位条目的 diff/apply 语义冲突
回代(41 条全部接受, 校验 0 错误):
- 西部牧场/铁道迷 五区: 普通档 7 项调慢、删 玻璃/杰皇 普通条目(改记为 SC);
  SC 档补齐 r兔/杰皇/黑龙/ssc/白龙/猫头鹰, 玻璃 22.34→22.09;
  五区高手补普通 r兔★6/c2★6/杰弟★6/21c★6/黑龙★6 + SC 21c★6/黑龙★6/白龙★6
- 狂野赛车场/极速前进: f5★6 38.7→24.5(上轮判定的漏改), 玻璃★6 微调 24.3,
  新增 cc850★6=24.9 / fe3★5=25.8; 四区高手 玻璃 由★6 改★3=24.8(修正星级越界) + fe3★5=25.8
- 冰火岛/地心探险: 上轮疑填错行的 万达★6=26.9 已归位到稳定跳图,
  并补 sgt★6=27.8 / 小牛★6=28.9; 旧跳图 sgt★6=22.9
- 高地穿梭/幽灵船: 9x8★6 22.9→22.75, 补 sf90★6=22.97 / 秋王★6=22.69
- 沙漠高速/发夹弯冲刺: 速尾★6=22.99

工具修复(apply_changes.py): SC 条目在 json 中常以"占位"形式存在
(有 car/sc_type 但无 time), 对应 xlsx 空单元格。填值时 diff 侧报
added+old_present=false, apply 侧却按"条目是否存在"判 true, 导致
"旧值不匹配"而卡死回代。现改为按"是否有 time"判定存在性, 与
"空单元格 = 无成绩"的口径对齐。补回归测试
test_sc_placeholder_fill_accepts_absent_old_and_keeps_route(21 项全绿)。

验证: 84 组同区同档同车同星配对 SC 全部快于普通(上轮 80 组, 0 违例),
中位提速 -0.45s; 理论->高手 SC 偏移 28 对中位 +0.30s;
两份 xlsx 已重导, 往返校验 0 值差异 0 结构差异。
特殊跑法四表列集保持按区档: 38/17/18/6, 理论表无带星列、高手表全带星。
</commit_message>
<xml_diff>
--- a/gauntlet_data.xlsx
+++ b/gauntlet_data.xlsx
@@ -30,9 +30,9 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'四区_普通'!$A$1:$BJ$84</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'四区_自动'!$A$1:$P$84</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'五区_理论_特殊跑法'!$A$1:$AO$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'五区_高手_特殊跑法'!$A$1:$R$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'五区_高手_特殊跑法'!$A$1:$T$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'四区_理论_特殊跑法'!$A$1:$U$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'四区_高手_特殊跑法'!$A$1:$G$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'四区_高手_特殊跑法'!$A$1:$I$21</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2739,12 +2739,8 @@
           <t>铁道迷</t>
         </is>
       </c>
-      <c r="C24" s="4" t="n">
-        <v>22.22</v>
-      </c>
-      <c r="D24" s="4" t="n">
-        <v>21.9</v>
-      </c>
+      <c r="C24" s="4" t="n"/>
+      <c r="D24" s="4" t="n"/>
       <c r="E24" s="4" t="n"/>
       <c r="F24" s="4" t="n">
         <v>21.5</v>
@@ -2753,24 +2749,24 @@
       <c r="H24" s="4" t="n"/>
       <c r="I24" s="4" t="n"/>
       <c r="J24" s="4" t="n">
-        <v>22.2</v>
+        <v>22.35</v>
       </c>
       <c r="K24" s="4" t="n"/>
       <c r="L24" s="4" t="n"/>
       <c r="M24" s="4" t="n">
-        <v>22.09</v>
+        <v>22.25</v>
       </c>
       <c r="N24" s="4" t="n"/>
       <c r="O24" s="4" t="n">
-        <v>22.11</v>
+        <v>22.32</v>
       </c>
       <c r="P24" s="4" t="n">
-        <v>22.5</v>
+        <v>22.57</v>
       </c>
       <c r="Q24" s="4" t="n"/>
       <c r="R24" s="4" t="n"/>
       <c r="S24" s="4" t="n">
-        <v>22.31</v>
+        <v>22.6</v>
       </c>
       <c r="T24" s="4" t="n"/>
       <c r="U24" s="4" t="n"/>
@@ -2783,13 +2779,13 @@
       <c r="Z24" s="4" t="n"/>
       <c r="AA24" s="4" t="n"/>
       <c r="AB24" s="4" t="n">
-        <v>22.45</v>
+        <v>22.62</v>
       </c>
       <c r="AC24" s="4" t="n"/>
       <c r="AD24" s="4" t="n"/>
       <c r="AE24" s="4" t="n"/>
       <c r="AF24" s="4" t="n">
-        <v>22.42</v>
+        <v>22.55</v>
       </c>
       <c r="AG24" s="4" t="n"/>
       <c r="AH24" s="4" t="n"/>
@@ -7750,7 +7746,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R21"/>
+  <dimension ref="A1:T21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -7771,6 +7767,8 @@
     <col width="7.5" customWidth="1" min="16" max="16"/>
     <col width="7.5" customWidth="1" min="17" max="17"/>
     <col width="7.5" customWidth="1" min="18" max="18"/>
+    <col width="7.5" customWidth="1" min="19" max="19"/>
+    <col width="7.5" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7816,50 +7814,60 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
+          <t>21c★6</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>9x8★6</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>黑龙★6</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>cc850★6</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>白龙★6</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>万达★6</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>速尾★6</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>sf90★6</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>sgt★6</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>秋王★6</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>小牛★6</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>fe3★5</t>
         </is>
@@ -7896,6 +7904,8 @@
       <c r="P2" s="4" t="n"/>
       <c r="Q2" s="4" t="n"/>
       <c r="R2" s="4" t="n"/>
+      <c r="S2" s="4" t="n"/>
+      <c r="T2" s="4" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="6" t="n"/>
@@ -7924,6 +7934,8 @@
       <c r="P3" s="4" t="n"/>
       <c r="Q3" s="4" t="n"/>
       <c r="R3" s="4" t="n"/>
+      <c r="S3" s="4" t="n"/>
+      <c r="T3" s="4" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -7960,6 +7972,8 @@
       <c r="P4" s="4" t="n"/>
       <c r="Q4" s="4" t="n"/>
       <c r="R4" s="4" t="n"/>
+      <c r="S4" s="4" t="n"/>
+      <c r="T4" s="4" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -7984,20 +7998,26 @@
       </c>
       <c r="G5" s="4" t="n"/>
       <c r="H5" s="4" t="n"/>
-      <c r="I5" s="4" t="n">
-        <v>22.9</v>
-      </c>
-      <c r="J5" s="4" t="n"/>
-      <c r="K5" s="4" t="n">
+      <c r="I5" s="4" t="n"/>
+      <c r="J5" s="4" t="n">
+        <v>22.75</v>
+      </c>
+      <c r="K5" s="4" t="n"/>
+      <c r="L5" s="4" t="n"/>
+      <c r="M5" s="4" t="n">
         <v>22.5</v>
       </c>
-      <c r="L5" s="4" t="n"/>
-      <c r="M5" s="4" t="n"/>
       <c r="N5" s="4" t="n"/>
       <c r="O5" s="4" t="n"/>
-      <c r="P5" s="4" t="n"/>
+      <c r="P5" s="4" t="n">
+        <v>22.97</v>
+      </c>
       <c r="Q5" s="4" t="n"/>
-      <c r="R5" s="4" t="n"/>
+      <c r="R5" s="4" t="n">
+        <v>22.69</v>
+      </c>
+      <c r="S5" s="4" t="n"/>
+      <c r="T5" s="4" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -8022,16 +8042,24 @@
       <c r="H6" s="4" t="n">
         <v>22.29</v>
       </c>
-      <c r="I6" s="4" t="n"/>
+      <c r="I6" s="4" t="n">
+        <v>22.19</v>
+      </c>
       <c r="J6" s="4" t="n"/>
-      <c r="K6" s="4" t="n"/>
+      <c r="K6" s="4" t="n">
+        <v>22.26</v>
+      </c>
       <c r="L6" s="4" t="n"/>
-      <c r="M6" s="4" t="n"/>
+      <c r="M6" s="4" t="n">
+        <v>22.5</v>
+      </c>
       <c r="N6" s="4" t="n"/>
       <c r="O6" s="4" t="n"/>
       <c r="P6" s="4" t="n"/>
       <c r="Q6" s="4" t="n"/>
       <c r="R6" s="4" t="n"/>
+      <c r="S6" s="4" t="n"/>
+      <c r="T6" s="4" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -8064,6 +8092,8 @@
       <c r="P7" s="4" t="n"/>
       <c r="Q7" s="4" t="n"/>
       <c r="R7" s="4" t="n"/>
+      <c r="S7" s="4" t="n"/>
+      <c r="T7" s="4" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -8095,11 +8125,13 @@
       <c r="M8" s="4" t="n"/>
       <c r="N8" s="4" t="n"/>
       <c r="O8" s="4" t="n"/>
-      <c r="P8" s="4" t="n">
+      <c r="P8" s="4" t="n"/>
+      <c r="Q8" s="4" t="n"/>
+      <c r="R8" s="4" t="n">
         <v>18.9</v>
       </c>
-      <c r="Q8" s="4" t="n"/>
-      <c r="R8" s="4" t="n"/>
+      <c r="S8" s="4" t="n"/>
+      <c r="T8" s="4" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -8132,6 +8164,8 @@
       <c r="P9" s="4" t="n"/>
       <c r="Q9" s="4" t="n"/>
       <c r="R9" s="4" t="n"/>
+      <c r="S9" s="4" t="n"/>
+      <c r="T9" s="4" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="6" t="n"/>
@@ -8160,6 +8194,8 @@
       <c r="P10" s="4" t="n"/>
       <c r="Q10" s="4" t="n"/>
       <c r="R10" s="4" t="n"/>
+      <c r="S10" s="4" t="n"/>
+      <c r="T10" s="4" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -8194,6 +8230,8 @@
       <c r="P11" s="4" t="n"/>
       <c r="Q11" s="4" t="n"/>
       <c r="R11" s="4" t="n"/>
+      <c r="S11" s="4" t="n"/>
+      <c r="T11" s="4" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -8222,10 +8260,14 @@
       <c r="L12" s="4" t="n"/>
       <c r="M12" s="4" t="n"/>
       <c r="N12" s="4" t="n"/>
-      <c r="O12" s="4" t="n"/>
+      <c r="O12" s="4" t="n">
+        <v>22.99</v>
+      </c>
       <c r="P12" s="4" t="n"/>
       <c r="Q12" s="4" t="n"/>
       <c r="R12" s="4" t="n"/>
+      <c r="S12" s="4" t="n"/>
+      <c r="T12" s="4" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -8258,6 +8300,8 @@
       <c r="P13" s="4" t="n"/>
       <c r="Q13" s="4" t="n"/>
       <c r="R13" s="4" t="n"/>
+      <c r="S13" s="4" t="n"/>
+      <c r="T13" s="4" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="6" t="n"/>
@@ -8272,24 +8316,30 @@
         </is>
       </c>
       <c r="D14" s="4" t="n">
-        <v>23.9</v>
+        <v>24.3</v>
       </c>
       <c r="E14" s="4" t="n"/>
       <c r="F14" s="4" t="n"/>
       <c r="G14" s="4" t="n">
-        <v>38.7</v>
+        <v>24.5</v>
       </c>
       <c r="H14" s="4" t="n"/>
       <c r="I14" s="4" t="n"/>
       <c r="J14" s="4" t="n"/>
       <c r="K14" s="4" t="n"/>
-      <c r="L14" s="4" t="n"/>
+      <c r="L14" s="4" t="n">
+        <v>24.9</v>
+      </c>
       <c r="M14" s="4" t="n"/>
       <c r="N14" s="4" t="n"/>
       <c r="O14" s="4" t="n"/>
       <c r="P14" s="4" t="n"/>
       <c r="Q14" s="4" t="n"/>
       <c r="R14" s="4" t="n"/>
+      <c r="S14" s="4" t="n"/>
+      <c r="T14" s="4" t="n">
+        <v>25.8</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -8322,6 +8372,8 @@
       <c r="P15" s="4" t="n"/>
       <c r="Q15" s="4" t="n"/>
       <c r="R15" s="4" t="n"/>
+      <c r="S15" s="4" t="n"/>
+      <c r="T15" s="4" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="n"/>
@@ -8348,8 +8400,12 @@
       <c r="N16" s="4" t="n"/>
       <c r="O16" s="4" t="n"/>
       <c r="P16" s="4" t="n"/>
-      <c r="Q16" s="4" t="n"/>
+      <c r="Q16" s="4" t="n">
+        <v>22.9</v>
+      </c>
       <c r="R16" s="4" t="n"/>
+      <c r="S16" s="4" t="n"/>
+      <c r="T16" s="4" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="n"/>
@@ -8373,11 +8429,19 @@
       <c r="K17" s="4" t="n"/>
       <c r="L17" s="4" t="n"/>
       <c r="M17" s="4" t="n"/>
-      <c r="N17" s="4" t="n"/>
+      <c r="N17" s="4" t="n">
+        <v>26.9</v>
+      </c>
       <c r="O17" s="4" t="n"/>
       <c r="P17" s="4" t="n"/>
-      <c r="Q17" s="4" t="n"/>
+      <c r="Q17" s="4" t="n">
+        <v>27.8</v>
+      </c>
       <c r="R17" s="4" t="n"/>
+      <c r="S17" s="4" t="n">
+        <v>28.9</v>
+      </c>
+      <c r="T17" s="4" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="6" t="n"/>
@@ -8406,6 +8470,8 @@
       <c r="P18" s="4" t="n"/>
       <c r="Q18" s="4" t="n"/>
       <c r="R18" s="4" t="n"/>
+      <c r="S18" s="4" t="n"/>
+      <c r="T18" s="4" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -8438,6 +8504,8 @@
       <c r="P19" s="4" t="n"/>
       <c r="Q19" s="4" t="n"/>
       <c r="R19" s="4" t="n"/>
+      <c r="S19" s="4" t="n"/>
+      <c r="T19" s="4" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -8462,18 +8530,20 @@
       <c r="H20" s="4" t="n"/>
       <c r="I20" s="4" t="n"/>
       <c r="J20" s="4" t="n"/>
-      <c r="K20" s="4" t="n">
+      <c r="K20" s="4" t="n"/>
+      <c r="L20" s="4" t="n"/>
+      <c r="M20" s="4" t="n">
         <v>18.6</v>
       </c>
-      <c r="L20" s="4" t="n"/>
-      <c r="M20" s="4" t="n"/>
       <c r="N20" s="4" t="n"/>
-      <c r="O20" s="4" t="n">
+      <c r="O20" s="4" t="n"/>
+      <c r="P20" s="4" t="n"/>
+      <c r="Q20" s="4" t="n">
         <v>18.9</v>
       </c>
-      <c r="P20" s="4" t="n"/>
-      <c r="Q20" s="4" t="n"/>
       <c r="R20" s="4" t="n"/>
+      <c r="S20" s="4" t="n"/>
+      <c r="T20" s="4" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -8508,9 +8578,11 @@
       <c r="P21" s="4" t="n"/>
       <c r="Q21" s="4" t="n"/>
       <c r="R21" s="4" t="n"/>
+      <c r="S21" s="4" t="n"/>
+      <c r="T21" s="4" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R21"/>
+  <autoFilter ref="A1:T21"/>
   <mergeCells count="14">
     <mergeCell ref="A8"/>
     <mergeCell ref="A6"/>
@@ -9452,7 +9524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9462,6 +9534,8 @@
     <col width="7.5" customWidth="1" min="5" max="5"/>
     <col width="7.5" customWidth="1" min="6" max="6"/>
     <col width="7.5" customWidth="1" min="7" max="7"/>
+    <col width="7.5" customWidth="1" min="8" max="8"/>
+    <col width="7.5" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -9482,22 +9556,32 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>玻璃★3</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>9x8★6</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>c2★6</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>fp1★6</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>sgt★6</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>fe3★5</t>
         </is>
       </c>
     </row>
@@ -9521,6 +9605,8 @@
       <c r="E2" s="4" t="n"/>
       <c r="F2" s="4" t="n"/>
       <c r="G2" s="4" t="n"/>
+      <c r="H2" s="4" t="n"/>
+      <c r="I2" s="4" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="6" t="n"/>
@@ -9538,6 +9624,8 @@
       <c r="E3" s="4" t="n"/>
       <c r="F3" s="4" t="n"/>
       <c r="G3" s="4" t="n"/>
+      <c r="H3" s="4" t="n"/>
+      <c r="I3" s="4" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -9557,10 +9645,12 @@
       </c>
       <c r="D4" s="4" t="n"/>
       <c r="E4" s="4" t="n"/>
-      <c r="F4" s="4" t="n">
+      <c r="F4" s="4" t="n"/>
+      <c r="G4" s="4" t="n">
         <v>24.79</v>
       </c>
-      <c r="G4" s="4" t="n"/>
+      <c r="H4" s="4" t="n"/>
+      <c r="I4" s="4" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -9578,12 +9668,14 @@
           <t>跳船</t>
         </is>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="D5" s="4" t="n"/>
+      <c r="E5" s="4" t="n">
         <v>22.9</v>
       </c>
-      <c r="E5" s="4" t="n"/>
       <c r="F5" s="4" t="n"/>
       <c r="G5" s="4" t="n"/>
+      <c r="H5" s="4" t="n"/>
+      <c r="I5" s="4" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -9602,11 +9694,13 @@
         </is>
       </c>
       <c r="D6" s="4" t="n"/>
-      <c r="E6" s="4" t="n">
+      <c r="E6" s="4" t="n"/>
+      <c r="F6" s="4" t="n">
         <v>22.6</v>
       </c>
-      <c r="F6" s="4" t="n"/>
       <c r="G6" s="4" t="n"/>
+      <c r="H6" s="4" t="n"/>
+      <c r="I6" s="4" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -9628,6 +9722,8 @@
       <c r="E7" s="4" t="n"/>
       <c r="F7" s="4" t="n"/>
       <c r="G7" s="4" t="n"/>
+      <c r="H7" s="4" t="n"/>
+      <c r="I7" s="4" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -9649,6 +9745,8 @@
       <c r="E8" s="4" t="n"/>
       <c r="F8" s="4" t="n"/>
       <c r="G8" s="4" t="n"/>
+      <c r="H8" s="4" t="n"/>
+      <c r="I8" s="4" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -9670,6 +9768,8 @@
       <c r="E9" s="4" t="n"/>
       <c r="F9" s="4" t="n"/>
       <c r="G9" s="4" t="n"/>
+      <c r="H9" s="4" t="n"/>
+      <c r="I9" s="4" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="6" t="n"/>
@@ -9687,6 +9787,8 @@
       <c r="E10" s="4" t="n"/>
       <c r="F10" s="4" t="n"/>
       <c r="G10" s="4" t="n"/>
+      <c r="H10" s="4" t="n"/>
+      <c r="I10" s="4" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -9708,6 +9810,8 @@
       <c r="E11" s="4" t="n"/>
       <c r="F11" s="4" t="n"/>
       <c r="G11" s="4" t="n"/>
+      <c r="H11" s="4" t="n"/>
+      <c r="I11" s="4" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -9729,6 +9833,8 @@
       <c r="E12" s="4" t="n"/>
       <c r="F12" s="4" t="n"/>
       <c r="G12" s="4" t="n"/>
+      <c r="H12" s="4" t="n"/>
+      <c r="I12" s="4" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -9750,6 +9856,8 @@
       <c r="E13" s="4" t="n"/>
       <c r="F13" s="4" t="n"/>
       <c r="G13" s="4" t="n"/>
+      <c r="H13" s="4" t="n"/>
+      <c r="I13" s="4" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="6" t="n"/>
@@ -9763,10 +9871,16 @@
           <t>跳图</t>
         </is>
       </c>
-      <c r="D14" s="4" t="n"/>
+      <c r="D14" s="4" t="n">
+        <v>24.8</v>
+      </c>
       <c r="E14" s="4" t="n"/>
       <c r="F14" s="4" t="n"/>
       <c r="G14" s="4" t="n"/>
+      <c r="H14" s="4" t="n"/>
+      <c r="I14" s="4" t="n">
+        <v>25.8</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -9788,6 +9902,8 @@
       <c r="E15" s="4" t="n"/>
       <c r="F15" s="4" t="n"/>
       <c r="G15" s="4" t="n"/>
+      <c r="H15" s="4" t="n"/>
+      <c r="I15" s="4" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="n"/>
@@ -9805,6 +9921,8 @@
       <c r="E16" s="4" t="n"/>
       <c r="F16" s="4" t="n"/>
       <c r="G16" s="4" t="n"/>
+      <c r="H16" s="4" t="n"/>
+      <c r="I16" s="4" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="n"/>
@@ -9822,6 +9940,8 @@
       <c r="E17" s="4" t="n"/>
       <c r="F17" s="4" t="n"/>
       <c r="G17" s="4" t="n"/>
+      <c r="H17" s="4" t="n"/>
+      <c r="I17" s="4" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="6" t="n"/>
@@ -9839,6 +9959,8 @@
       <c r="E18" s="4" t="n"/>
       <c r="F18" s="4" t="n"/>
       <c r="G18" s="4" t="n"/>
+      <c r="H18" s="4" t="n"/>
+      <c r="I18" s="4" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -9860,6 +9982,8 @@
       <c r="E19" s="4" t="n"/>
       <c r="F19" s="4" t="n"/>
       <c r="G19" s="4" t="n"/>
+      <c r="H19" s="4" t="n"/>
+      <c r="I19" s="4" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -9880,9 +10004,11 @@
       <c r="D20" s="4" t="n"/>
       <c r="E20" s="4" t="n"/>
       <c r="F20" s="4" t="n"/>
-      <c r="G20" s="4" t="n">
+      <c r="G20" s="4" t="n"/>
+      <c r="H20" s="4" t="n">
         <v>18.9</v>
       </c>
+      <c r="I20" s="4" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -9904,9 +10030,11 @@
       <c r="E21" s="4" t="n"/>
       <c r="F21" s="4" t="n"/>
       <c r="G21" s="4" t="n"/>
+      <c r="H21" s="4" t="n"/>
+      <c r="I21" s="4" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G21"/>
+  <autoFilter ref="A1:I21"/>
   <mergeCells count="14">
     <mergeCell ref="A8"/>
     <mergeCell ref="A6"/>
@@ -12874,7 +13002,9 @@
       <c r="K24" s="4" t="n"/>
       <c r="L24" s="4" t="n"/>
       <c r="M24" s="4" t="n"/>
-      <c r="N24" s="4" t="n"/>
+      <c r="N24" s="4" t="n">
+        <v>21.87</v>
+      </c>
       <c r="O24" s="4" t="n"/>
       <c r="P24" s="4" t="n"/>
       <c r="Q24" s="4" t="n"/>
@@ -12884,14 +13014,22 @@
       <c r="U24" s="4" t="n"/>
       <c r="V24" s="4" t="n"/>
       <c r="W24" s="4" t="n"/>
-      <c r="X24" s="4" t="n"/>
-      <c r="Y24" s="4" t="n"/>
+      <c r="X24" s="4" t="n">
+        <v>22.43</v>
+      </c>
+      <c r="Y24" s="4" t="n">
+        <v>22.45</v>
+      </c>
       <c r="Z24" s="4" t="n"/>
       <c r="AA24" s="4" t="n"/>
       <c r="AB24" s="4" t="n"/>
-      <c r="AC24" s="4" t="n"/>
+      <c r="AC24" s="4" t="n">
+        <v>22.39</v>
+      </c>
       <c r="AD24" s="4" t="n"/>
-      <c r="AE24" s="4" t="n"/>
+      <c r="AE24" s="4" t="n">
+        <v>22.47</v>
+      </c>
       <c r="AF24" s="4" t="n"/>
       <c r="AG24" s="4" t="n"/>
       <c r="AH24" s="4" t="n"/>
@@ -62126,11 +62264,15 @@
         </is>
       </c>
       <c r="D6" s="4" t="n">
-        <v>22.34</v>
-      </c>
-      <c r="E6" s="4" t="n"/>
+        <v>22.09</v>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>21.9</v>
+      </c>
       <c r="F6" s="4" t="n"/>
-      <c r="G6" s="4" t="n"/>
+      <c r="G6" s="4" t="n">
+        <v>21.49</v>
+      </c>
       <c r="H6" s="4" t="n"/>
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="4" t="n"/>
@@ -62147,12 +62289,18 @@
       <c r="O6" s="4" t="n">
         <v>23.58</v>
       </c>
-      <c r="P6" s="4" t="n"/>
-      <c r="Q6" s="4" t="n"/>
+      <c r="P6" s="4" t="n">
+        <v>22.14</v>
+      </c>
+      <c r="Q6" s="4" t="n">
+        <v>22.39</v>
+      </c>
       <c r="R6" s="4" t="n">
         <v>21.95</v>
       </c>
-      <c r="S6" s="4" t="n"/>
+      <c r="S6" s="4" t="n">
+        <v>22.3</v>
+      </c>
       <c r="T6" s="4" t="n"/>
       <c r="U6" s="4" t="n"/>
       <c r="V6" s="4" t="n"/>
@@ -62160,7 +62308,9 @@
       <c r="X6" s="4" t="n"/>
       <c r="Y6" s="4" t="n"/>
       <c r="Z6" s="4" t="n"/>
-      <c r="AA6" s="4" t="n"/>
+      <c r="AA6" s="4" t="n">
+        <v>22.42</v>
+      </c>
       <c r="AB6" s="4" t="n">
         <v>23.11</v>
       </c>
@@ -62856,18 +63006,20 @@
       <c r="W17" s="4" t="n"/>
       <c r="X17" s="4" t="n"/>
       <c r="Y17" s="4" t="n">
-        <v>28</v>
+        <v>27.5</v>
       </c>
       <c r="Z17" s="4" t="n"/>
       <c r="AA17" s="4" t="n"/>
       <c r="AB17" s="4" t="n"/>
       <c r="AC17" s="4" t="n"/>
       <c r="AD17" s="4" t="n">
-        <v>29</v>
+        <v>28.5</v>
       </c>
       <c r="AE17" s="4" t="n"/>
       <c r="AF17" s="4" t="n"/>
-      <c r="AG17" s="4" t="n"/>
+      <c r="AG17" s="4" t="n">
+        <v>27.9</v>
+      </c>
       <c r="AH17" s="4" t="n"/>
       <c r="AI17" s="4" t="n"/>
       <c r="AJ17" s="4" t="n"/>

</xml_diff>